<commit_message>
Export XLSX from Google Sheet (entities)
</commit_message>
<xml_diff>
--- a/gsheet/xlsx/entities.xlsx
+++ b/gsheet/xlsx/entities.xlsx
@@ -3974,10 +3974,10 @@
     <t>place_058</t>
   </si>
   <si>
-    <t>Thurn/ genennt von Geissen</t>
-  </si>
-  <si>
-    <t>ein Turm?</t>
+    <t>Geissturm</t>
+  </si>
+  <si>
+    <t>Pulverturm</t>
   </si>
   <si>
     <t>place_059</t>
@@ -14977,7 +14977,7 @@
       </c>
       <c r="B59" s="24" t="str">
         <f t="shared" si="1"/>
-        <v>Thurn/ genennt von Geissen</v>
+        <v>Geissturm</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>1273</v>

</xml_diff>